<commit_message>
Sprint 11: marcar RF-071 a RF-077 como concluídos no backlog
Somente a coluna Status das sete linhas da Sprint 11, com o vocabulário já
usado na planilha. Backup do arquivo original em docs/backup/.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -7521,7 +7521,7 @@
         <v>236</v>
       </c>
       <c r="I82" s="6" t="s">
-        <v>54</v>
+        <v>431</v>
       </c>
       <c r="J82" s="6" t="s">
         <v>134</v>
@@ -7556,7 +7556,7 @@
         <v>236</v>
       </c>
       <c r="I83" s="6" t="s">
-        <v>54</v>
+        <v>431</v>
       </c>
       <c r="J83" s="6" t="s">
         <v>134</v>
@@ -7591,7 +7591,7 @@
         <v>236</v>
       </c>
       <c r="I84" s="6" t="s">
-        <v>54</v>
+        <v>431</v>
       </c>
       <c r="J84" s="6" t="s">
         <v>134</v>
@@ -7626,7 +7626,7 @@
         <v>236</v>
       </c>
       <c r="I85" s="6" t="s">
-        <v>54</v>
+        <v>431</v>
       </c>
       <c r="J85" s="6" t="s">
         <v>134</v>
@@ -7661,7 +7661,7 @@
         <v>236</v>
       </c>
       <c r="I86" s="6" t="s">
-        <v>54</v>
+        <v>431</v>
       </c>
       <c r="J86" s="6" t="s">
         <v>134</v>
@@ -7696,7 +7696,7 @@
         <v>236</v>
       </c>
       <c r="I87" s="6" t="s">
-        <v>54</v>
+        <v>431</v>
       </c>
       <c r="J87" s="6" t="s">
         <v>134</v>
@@ -7731,7 +7731,7 @@
         <v>236</v>
       </c>
       <c r="I88" s="6" t="s">
-        <v>54</v>
+        <v>431</v>
       </c>
       <c r="J88" s="6" t="s">
         <v>134</v>

</xml_diff>

<commit_message>
Front end sprint 18
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -9629,7 +9629,7 @@
       </c>
       <c r="I134" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J134" s="6" t="inlineStr">
@@ -9684,7 +9684,7 @@
       </c>
       <c r="I135" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J135" s="6" t="inlineStr">
@@ -9739,7 +9739,7 @@
       </c>
       <c r="I136" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J136" s="6" t="inlineStr">
@@ -9794,7 +9794,7 @@
       </c>
       <c r="I137" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J137" s="6" t="inlineStr">
@@ -9849,7 +9849,7 @@
       </c>
       <c r="I138" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J138" s="6" t="inlineStr">
@@ -9904,7 +9904,7 @@
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J139" s="6" t="inlineStr">

</xml_diff>

<commit_message>
UI-035: histórico de compras e evolução de preços; rotas e testes do módulo Compras
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -11224,7 +11224,7 @@
       </c>
       <c r="I163" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J163" s="6" t="inlineStr">
@@ -11279,7 +11279,7 @@
       </c>
       <c r="I164" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J164" s="6" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="I165" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J165" s="6" t="inlineStr">
@@ -11389,7 +11389,7 @@
       </c>
       <c r="I166" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J166" s="6" t="inlineStr">
@@ -11444,7 +11444,7 @@
       </c>
       <c r="I167" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J167" s="6" t="inlineStr">
@@ -11499,7 +11499,7 @@
       </c>
       <c r="I168" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J168" s="6" t="inlineStr">

</xml_diff>

<commit_message>
UI-053: histórico de conciliações e trilha de desfazimento; testes e backlog da Sprint 26
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -12214,7 +12214,7 @@
       </c>
       <c r="I181" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J181" s="6" t="inlineStr">
@@ -12269,7 +12269,7 @@
       </c>
       <c r="I182" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J182" s="6" t="inlineStr">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="I183" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J183" s="6" t="inlineStr">
@@ -12379,7 +12379,7 @@
       </c>
       <c r="I184" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J184" s="6" t="inlineStr">
@@ -12434,7 +12434,7 @@
       </c>
       <c r="I185" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J185" s="6" t="inlineStr">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="I186" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J186" s="6" t="inlineStr">

</xml_diff>

<commit_message>
UI-060: exportação contábil; rotas, testes e backlog da Sprint 27
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -12544,7 +12544,7 @@
       </c>
       <c r="I187" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J187" s="6" t="inlineStr">
@@ -12599,7 +12599,7 @@
       </c>
       <c r="I188" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J188" s="6" t="inlineStr">
@@ -12654,7 +12654,7 @@
       </c>
       <c r="I189" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J189" s="6" t="inlineStr">
@@ -12709,7 +12709,7 @@
       </c>
       <c r="I190" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J190" s="6" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="I191" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J191" s="6" t="inlineStr">
@@ -12819,7 +12819,7 @@
       </c>
       <c r="I192" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J192" s="6" t="inlineStr">
@@ -12874,7 +12874,7 @@
       </c>
       <c r="I193" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J193" s="6" t="inlineStr">

</xml_diff>

<commit_message>
UI-067: editor de regras de automação com condições, ações e histórico
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -12929,7 +12929,7 @@
       </c>
       <c r="I194" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J194" s="6" t="inlineStr">
@@ -12984,7 +12984,7 @@
       </c>
       <c r="I195" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J195" s="6" t="inlineStr">
@@ -13039,7 +13039,7 @@
       </c>
       <c r="I196" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J196" s="6" t="inlineStr">
@@ -13094,7 +13094,7 @@
       </c>
       <c r="I197" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J197" s="6" t="inlineStr">
@@ -13149,7 +13149,7 @@
       </c>
       <c r="I198" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J198" s="6" t="inlineStr">
@@ -13204,7 +13204,7 @@
       </c>
       <c r="I199" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J199" s="6" t="inlineStr">
@@ -13259,7 +13259,7 @@
       </c>
       <c r="I200" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J200" s="6" t="inlineStr">

</xml_diff>

<commit_message>
UI-075: monitoramento de integrações, diário de erros e reprocessamento
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -13314,7 +13314,7 @@
       </c>
       <c r="I201" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J201" s="6" t="inlineStr">
@@ -13369,7 +13369,7 @@
       </c>
       <c r="I202" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J202" s="6" t="inlineStr">
@@ -13424,7 +13424,7 @@
       </c>
       <c r="I203" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J203" s="6" t="inlineStr">
@@ -13479,7 +13479,7 @@
       </c>
       <c r="I204" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J204" s="6" t="inlineStr">
@@ -13534,7 +13534,7 @@
       </c>
       <c r="I205" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J205" s="6" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="I206" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J206" s="6" t="inlineStr">
@@ -13644,7 +13644,7 @@
       </c>
       <c r="I207" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J207" s="6" t="inlineStr">
@@ -13699,7 +13699,7 @@
       </c>
       <c r="I208" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J208" s="6" t="inlineStr">

</xml_diff>

<commit_message>
UI-076 a UI-081: design system vivo, busca global, preferências, onboarding, impressão/exportação e estados padronizados
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -13752,10 +13752,8 @@
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="I209" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A Fazer</t>
-        </is>
+      <c r="I209" s="6" t="s">
+        <v>431</v>
       </c>
       <c r="J209" s="6" t="inlineStr">
         <is>
@@ -13807,10 +13805,8 @@
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="I210" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A Fazer</t>
-        </is>
+      <c r="I210" s="6" t="s">
+        <v>431</v>
       </c>
       <c r="J210" s="6" t="inlineStr">
         <is>
@@ -13862,10 +13858,8 @@
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="I211" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A Fazer</t>
-        </is>
+      <c r="I211" s="6" t="s">
+        <v>431</v>
       </c>
       <c r="J211" s="6" t="inlineStr">
         <is>
@@ -13917,10 +13911,8 @@
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="I212" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A Fazer</t>
-        </is>
+      <c r="I212" s="6" t="s">
+        <v>431</v>
       </c>
       <c r="J212" s="6" t="inlineStr">
         <is>
@@ -13972,10 +13964,8 @@
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="I213" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A Fazer</t>
-        </is>
+      <c r="I213" s="6" t="s">
+        <v>431</v>
       </c>
       <c r="J213" s="6" t="inlineStr">
         <is>
@@ -14027,10 +14017,8 @@
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="I214" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A Fazer</t>
-        </is>
+      <c r="I214" s="6" t="s">
+        <v>431</v>
       </c>
       <c r="J214" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
UI-082 a UI-086: acessibilidade WCAG 2.1 AA, responsividade, formatos pt-BR, cache e virtualização, auditoria de interface
</commit_message>
<xml_diff>
--- a/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
+++ b/docs/Sprints_Sistema_Gestao_Empresarial_Financeira.xlsx
@@ -1,21 +1,25 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
-  <sheets>
-    <sheet state="visible" name="Resumo do Projeto" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Visão Geral das Sprints" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Backlog de Sprints" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Legenda" sheetId="4" r:id="rId8"/>
-  </sheets>
-  <definedNames>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Backlog de Sprints'!$A$1:$K$132</definedName>
-  </definedNames>
-  <calcPr/>
-</workbook>
+<file path=xl\drawings\drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\drawings\drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl\drawings\drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl\drawings\drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl\persons\person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1501" uniqueCount="432">
   <si>
     <t>Planejamento de Sprints</t>
@@ -1316,7 +1320,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <fonts count="7">
     <font>
@@ -1439,27 +1443,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
@@ -1653,7 +1637,23 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <workbookPr/>
+  <sheets>
+    <sheet state="visible" name="Resumo do Projeto" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Visão Geral das Sprints" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="Backlog de Sprints" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Legenda" sheetId="4" r:id="rId8"/>
+  </sheets>
+  <definedNames>
+    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Backlog de Sprints'!$A$1:$K$132</definedName>
+  </definedNames>
+  <calcPr/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>
@@ -2908,7 +2908,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>
@@ -4948,7 +4948,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>
@@ -14072,7 +14072,7 @@
       </c>
       <c r="I215" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J215" s="6" t="inlineStr">
@@ -14127,7 +14127,7 @@
       </c>
       <c r="I216" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J216" s="6" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="I217" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J217" s="6" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="I218" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J218" s="6" t="inlineStr">
@@ -14292,7 +14292,7 @@
       </c>
       <c r="I219" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Fazer</t>
+          <t xml:space="preserve">Concluído</t>
         </is>
       </c>
       <c r="J219" s="6" t="inlineStr">
@@ -15474,7 +15474,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>

</xml_diff>